<commit_message>
upload cost factors and fixed how to compute MAC sign correctly
</commit_message>
<xml_diff>
--- a/ssp_modeling/cost-benefits/tornado_plot/data/output/tornado_plot_for_QA_for_edmundo_jan_21.xlsx
+++ b/ssp_modeling/cost-benefits/tornado_plot/data/output/tornado_plot_for_QA_for_edmundo_jan_21.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10110"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10125"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tony/Documents/sisepuede_modeling/ssp_bulgaria/ssp_modeling/cost-benefits/tornado_plot/data/output/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E521DFAE-67FB-554D-B576-E7F6D25A94A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EECF3AAA-24C1-9843-B2B6-EA39317EEBE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6540" yWindow="22260" windowWidth="30240" windowHeight="18980" xr2:uid="{280C43B5-CAFF-4743-A421-21B105102BCB}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="19680" xr2:uid="{280C43B5-CAFF-4743-A421-21B105102BCB}"/>
   </bookViews>
   <sheets>
     <sheet name="tornado_plot_for_QA_stable" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">tornado_plot_for_QA_stable!$A$1:$K$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">tornado_plot_for_QA_stable!$A$1:$K$21</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="98">
   <si>
     <t>transformation_name</t>
   </si>
@@ -317,9 +317,6 @@
     <t>US EPA landfill gas collection/cost-effectiveness doc. (US EPA)</t>
   </si>
   <si>
-    <t>Low-to-moderate cost; can become cost-saving with revenue streams (energy, fertilizer)</t>
-  </si>
-  <si>
     <t>Same: depends on scale/system boundary</t>
   </si>
   <si>
@@ -525,24 +522,12 @@
     <t>https://www.oecd.org/content/dam/oecd/en/publications/reports/2015/08/cost-effectiveness-of-greenhouse-gas-mitigation-measures-for-agriculture_g17a26e9/5jrvvkq900vj-en.pdf?utm_source=chatgpt.com</t>
   </si>
   <si>
-    <t>−15 to +60</t>
-  </si>
-  <si>
-    <t>−40 to +20</t>
-  </si>
-  <si>
-    <t>−10 to +30</t>
-  </si>
-  <si>
     <t>–50 to +80</t>
   </si>
   <si>
     <t>https://climate.ec.europa.eu/system/files/2016-11/ir_07_nonco2_en.pdf?utm_source=chatgpt.com</t>
   </si>
   <si>
-    <t>−50 to +20</t>
-  </si>
-  <si>
     <t>https://www.ipcc.ch/report/ar6/wg3/downloads/report/IPCC_AR6_WGIII_Chapter11.pdf</t>
   </si>
   <si>
@@ -555,9 +540,6 @@
     <t>WASO actions to increase and capture biogas</t>
   </si>
   <si>
-    <t>Increase biogas capture</t>
-  </si>
-  <si>
     <t>Improved rural wastewater treatment</t>
   </si>
   <si>
@@ -571,6 +553,24 @@
   </si>
   <si>
     <t>https://www.ipcc-nggip.iges.or.jp/public/2019rf/pdf/5_Volume5/19R_V5_6_Ch06_Wastewater.pdf?utm_source=chatgpt.com</t>
+  </si>
+  <si>
+    <t>Industrial carbon capture and sequestration</t>
+  </si>
+  <si>
+    <t>Increase solid waste biogas capture</t>
+  </si>
+  <si>
+    <t>–30 to +40</t>
+  </si>
+  <si>
+    <t>5 to 30</t>
+  </si>
+  <si>
+    <t>20 to 60</t>
+  </si>
+  <si>
+    <t>moderate cost</t>
   </si>
 </sst>
 </file>
@@ -578,7 +578,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="0.0000"/>
+    <numFmt numFmtId="164" formatCode="0.0000"/>
   </numFmts>
   <fonts count="22" x14ac:knownFonts="1">
     <font>
@@ -1104,8 +1104,8 @@
     <xf numFmtId="0" fontId="21" fillId="33" borderId="0" xfId="42" applyFill="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="165" fontId="0" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1482,7 +1482,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D3910A4A-016A-C04F-9DC6-2D7CC5B9E4C9}">
-  <dimension ref="A1:K24"/>
+  <dimension ref="A1:K25"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="51.6640625" bestFit="1" customWidth="1"/>
@@ -1520,7 +1520,7 @@
         <v>6</v>
       </c>
       <c r="H1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>33</v>
@@ -1532,44 +1532,35 @@
         <v>35</v>
       </c>
     </row>
-    <row r="2" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C2" s="7">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>92</v>
+      </c>
+      <c r="B2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C2" s="6">
         <v>135.46160097665</v>
       </c>
-      <c r="D2" s="7">
-        <v>134.526573707209</v>
-      </c>
-      <c r="E2" s="7">
-        <v>-0.93502726944063796</v>
-      </c>
-      <c r="F2" s="9">
-        <v>2.2323112282622799E-2</v>
-      </c>
-      <c r="G2" s="7">
-        <v>23.874290100626901</v>
-      </c>
-      <c r="H2" s="2">
-        <v>1</v>
-      </c>
-      <c r="I2" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="J2" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="K2" s="5" t="s">
-        <v>76</v>
-      </c>
+      <c r="D2" s="6">
+        <v>92.834280587011506</v>
+      </c>
+      <c r="E2" s="6">
+        <v>-42.627320389638797</v>
+      </c>
+      <c r="F2" s="8">
+        <v>1.8622816137780001</v>
+      </c>
+      <c r="G2" s="6">
+        <v>43.687513002357498</v>
+      </c>
+      <c r="I2" s="1"/>
+      <c r="J2" s="1"/>
+      <c r="K2" s="1"/>
     </row>
     <row r="3" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>9</v>
@@ -1578,752 +1569,787 @@
         <v>135.46160097665</v>
       </c>
       <c r="D3" s="7">
-        <v>131.69765456751799</v>
+        <v>134.526573707209</v>
       </c>
       <c r="E3" s="7">
-        <v>-3.7639464091322998</v>
+        <v>-0.93502726944063796</v>
       </c>
       <c r="F3" s="9">
-        <v>6.6341437050231294E-2</v>
+        <v>2.2323112282622799E-2</v>
       </c>
       <c r="G3" s="7">
-        <v>17.625499897998001</v>
+        <v>23.874290100626901</v>
       </c>
       <c r="H3" s="2">
         <v>1</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>39</v>
+        <v>73</v>
       </c>
       <c r="J3" s="4" t="s">
-        <v>40</v>
+        <v>74</v>
       </c>
       <c r="K3" s="5" t="s">
-        <v>41</v>
+        <v>75</v>
       </c>
     </row>
     <row r="4" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="C4" s="7">
         <v>135.46160097665</v>
       </c>
       <c r="D4" s="7">
-        <v>134.75532875432401</v>
+        <v>131.69765456751799</v>
       </c>
       <c r="E4" s="7">
-        <v>-0.70627222232533804</v>
+        <v>-3.7639464091322998</v>
       </c>
       <c r="F4" s="9">
-        <v>-2.373569330875E-2</v>
+        <v>6.6341437050231294E-2</v>
       </c>
       <c r="G4" s="7">
-        <v>-33.607003869701003</v>
+        <v>17.625499897998001</v>
       </c>
       <c r="H4" s="2">
         <v>1</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>83</v>
+        <v>39</v>
       </c>
       <c r="J4" s="4" t="s">
-        <v>58</v>
+        <v>40</v>
       </c>
       <c r="K4" s="5" t="s">
-        <v>81</v>
+        <v>41</v>
       </c>
     </row>
     <row r="5" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="C5" s="7">
         <v>135.46160097665</v>
       </c>
       <c r="D5" s="7">
-        <v>135.06579988722001</v>
+        <v>134.75532875432401</v>
       </c>
       <c r="E5" s="7">
-        <v>-0.39580108942968101</v>
+        <v>-0.70627222232533804</v>
       </c>
       <c r="F5" s="9">
-        <v>5.1951858468603004E-3</v>
+        <v>2.373569330875E-2</v>
       </c>
       <c r="G5" s="7">
-        <v>13.1257492351679</v>
+        <v>33.607003869701003</v>
       </c>
       <c r="H5" s="2">
         <v>1</v>
       </c>
       <c r="I5" s="3" t="s">
-        <v>67</v>
+        <v>96</v>
       </c>
       <c r="J5" s="4" t="s">
-        <v>68</v>
+        <v>97</v>
       </c>
       <c r="K5" s="5" t="s">
-        <v>69</v>
+        <v>80</v>
       </c>
     </row>
     <row r="6" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C6" s="7">
         <v>135.46160097665</v>
       </c>
       <c r="D6" s="7">
-        <v>134.26802387902899</v>
+        <v>135.06579988722001</v>
       </c>
       <c r="E6" s="7">
-        <v>-1.1935770976204401</v>
+        <v>-0.39580108942968101</v>
       </c>
       <c r="F6" s="9">
-        <v>-0.22482639096818999</v>
+        <v>5.1951858468603004E-3</v>
       </c>
       <c r="G6" s="7">
-        <v>-188.363526257676</v>
+        <v>13.1257492351679</v>
       </c>
       <c r="H6" s="2">
         <v>1</v>
       </c>
       <c r="I6" s="3" t="s">
-        <v>36</v>
+        <v>66</v>
       </c>
       <c r="J6" s="4" t="s">
-        <v>37</v>
+        <v>67</v>
       </c>
       <c r="K6" s="5" t="s">
-        <v>38</v>
+        <v>68</v>
       </c>
     </row>
     <row r="7" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="C7" s="7">
         <v>135.46160097665</v>
       </c>
       <c r="D7" s="7">
-        <v>135.44577768712901</v>
+        <v>134.26802387902899</v>
       </c>
       <c r="E7" s="7">
-        <v>-1.58232895211654E-2</v>
+        <v>-1.1935770976204401</v>
       </c>
       <c r="F7" s="9">
-        <v>3.16465790422968E-4</v>
+        <v>-0.22482639096818999</v>
       </c>
       <c r="G7" s="7">
-        <v>19.999999999978499</v>
+        <v>-188.363526257676</v>
       </c>
       <c r="H7" s="2">
         <v>1</v>
       </c>
       <c r="I7" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="J7" s="4"/>
+        <v>36</v>
+      </c>
+      <c r="J7" s="4" t="s">
+        <v>37</v>
+      </c>
       <c r="K7" s="5" t="s">
-        <v>90</v>
+        <v>38</v>
       </c>
     </row>
     <row r="8" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="C8" s="7">
         <v>135.46160097665</v>
       </c>
       <c r="D8" s="7">
-        <v>135.32341644419299</v>
+        <v>135.44577768712901</v>
       </c>
       <c r="E8" s="7">
-        <v>-0.13818453245639201</v>
+        <v>-1.58232895211654E-2</v>
       </c>
       <c r="F8" s="9">
-        <v>8.9352764531657903E-3</v>
+        <v>3.16465790422968E-4</v>
       </c>
       <c r="G8" s="7">
-        <v>64.661914718896099</v>
+        <v>19.999999999978499</v>
       </c>
       <c r="H8" s="2">
         <v>1</v>
       </c>
       <c r="I8" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="J8" s="4" t="s">
-        <v>73</v>
-      </c>
+        <v>84</v>
+      </c>
+      <c r="J8" s="4"/>
       <c r="K8" s="5" t="s">
-        <v>71</v>
+        <v>85</v>
       </c>
     </row>
     <row r="9" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C9" s="7">
         <v>135.46160097665</v>
       </c>
       <c r="D9" s="7">
-        <v>131.15138729527899</v>
+        <v>135.32341644419299</v>
       </c>
       <c r="E9" s="7">
-        <v>-4.3102136813707803</v>
+        <v>-0.13818453245639201</v>
       </c>
       <c r="F9" s="9">
-        <v>6.46532037851483E-2</v>
+        <v>8.9352764531657903E-3</v>
       </c>
       <c r="G9" s="7">
-        <v>14.999999666973901</v>
+        <v>64.661914718896099</v>
       </c>
       <c r="H9" s="2">
         <v>1</v>
       </c>
       <c r="I9" s="3" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="J9" s="4" t="s">
-        <v>62</v>
+        <v>72</v>
       </c>
       <c r="K9" s="5" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
     </row>
     <row r="10" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C10" s="7">
         <v>135.46160097665</v>
       </c>
       <c r="D10" s="7">
-        <v>134.16630924158599</v>
+        <v>131.15138729527899</v>
       </c>
       <c r="E10" s="7">
-        <v>-1.29529173506352</v>
+        <v>-4.3102136813707803</v>
       </c>
       <c r="F10" s="9">
-        <v>-0.25759428439457699</v>
+        <v>6.46532037851483E-2</v>
       </c>
       <c r="G10" s="7">
-        <v>-198.86970434652201</v>
+        <v>14.999999666973901</v>
       </c>
       <c r="H10" s="2">
         <v>1</v>
       </c>
       <c r="I10" s="3" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="J10" s="4" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="K10" s="5" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
     </row>
     <row r="11" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="C11" s="7">
         <v>135.46160097665</v>
       </c>
       <c r="D11" s="7">
-        <v>129.58819034254699</v>
+        <v>134.16630924158599</v>
       </c>
       <c r="E11" s="7">
-        <v>-5.87341063410266</v>
+        <v>-1.29529173506352</v>
       </c>
       <c r="F11" s="9">
-        <v>-8.5209609145833295E-2</v>
+        <v>-0.25759428439457699</v>
       </c>
       <c r="G11" s="7">
-        <v>-14.5076880290103</v>
+        <v>-198.86970434652201</v>
       </c>
       <c r="H11" s="2">
         <v>1</v>
       </c>
       <c r="I11" s="3" t="s">
-        <v>82</v>
+        <v>63</v>
       </c>
       <c r="J11" s="4" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="K11" s="5" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
     </row>
     <row r="12" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="C12" s="7">
         <v>135.46160097665</v>
       </c>
       <c r="D12" s="7">
-        <v>129.42343262830099</v>
+        <v>129.58819034254699</v>
       </c>
       <c r="E12" s="7">
-        <v>-6.0381683483488704</v>
+        <v>-5.87341063410266</v>
       </c>
       <c r="F12" s="9">
-        <v>0.278272382616368</v>
+        <v>8.5209609145833295E-2</v>
       </c>
       <c r="G12" s="7">
-        <v>46.085562137806399</v>
+        <v>14.5076880290103</v>
       </c>
       <c r="H12" s="2">
         <v>1</v>
       </c>
       <c r="I12" s="3" t="s">
-        <v>42</v>
+        <v>94</v>
       </c>
       <c r="J12" s="4" t="s">
-        <v>43</v>
+        <v>58</v>
       </c>
       <c r="K12" s="5" t="s">
-        <v>44</v>
+        <v>59</v>
       </c>
     </row>
     <row r="13" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="C13" s="7">
         <v>135.46160097665</v>
       </c>
       <c r="D13" s="7">
-        <v>134.82830707967699</v>
+        <v>129.42343262830099</v>
       </c>
       <c r="E13" s="7">
-        <v>-0.63329389697233296</v>
+        <v>-6.0381683483488704</v>
       </c>
       <c r="F13" s="9">
-        <v>-5.1597209993749999E-3</v>
+        <v>0.278272382616368</v>
       </c>
       <c r="G13" s="7">
-        <v>-8.1474352177444302</v>
+        <v>46.085562137806399</v>
       </c>
       <c r="H13" s="2">
         <v>1</v>
       </c>
       <c r="I13" s="3" t="s">
-        <v>84</v>
+        <v>42</v>
       </c>
       <c r="J13" s="4" t="s">
-        <v>59</v>
+        <v>43</v>
       </c>
       <c r="K13" s="5" t="s">
-        <v>60</v>
+        <v>44</v>
       </c>
     </row>
     <row r="14" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="C14" s="7">
         <v>135.46160097665</v>
       </c>
       <c r="D14" s="7">
-        <v>133.820856988489</v>
+        <v>134.82830707967699</v>
       </c>
       <c r="E14" s="7">
-        <v>-1.6407439881611701</v>
+        <v>-0.63329389697233296</v>
       </c>
       <c r="F14" s="9">
-        <v>-3.1995210583710401E-3</v>
+        <v>5.1597209993749999E-3</v>
       </c>
       <c r="G14" s="7">
-        <v>-1.95004283511459</v>
+        <v>8.1474352177444302</v>
       </c>
       <c r="H14" s="2">
         <v>1</v>
       </c>
-      <c r="I14" s="4" t="s">
-        <v>45</v>
+      <c r="I14" s="3" t="s">
+        <v>95</v>
       </c>
       <c r="J14" s="4" t="s">
-        <v>46</v>
+        <v>58</v>
       </c>
       <c r="K14" s="5" t="s">
-        <v>47</v>
+        <v>59</v>
       </c>
     </row>
     <row r="15" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="C15" s="7">
         <v>135.46160097665</v>
       </c>
       <c r="D15" s="7">
-        <v>134.374141664544</v>
+        <v>133.820856988489</v>
       </c>
       <c r="E15" s="7">
-        <v>-1.0874593121062599</v>
+        <v>-1.6407439881611701</v>
       </c>
       <c r="F15" s="9">
-        <v>1.4174868650294201E-2</v>
+        <v>-3.1995210583710401E-3</v>
       </c>
       <c r="G15" s="7">
-        <v>13.034849665169901</v>
+        <v>-1.95004283511459</v>
       </c>
       <c r="H15" s="2">
         <v>1</v>
       </c>
-      <c r="I15" s="3" t="s">
-        <v>48</v>
+      <c r="I15" s="4" t="s">
+        <v>45</v>
       </c>
       <c r="J15" s="4" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="K15" s="5" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
     </row>
     <row r="16" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>27</v>
+        <v>10</v>
       </c>
       <c r="C16" s="7">
         <v>135.46160097665</v>
       </c>
       <c r="D16" s="7">
-        <v>136.07723299629799</v>
+        <v>134.374141664544</v>
       </c>
       <c r="E16" s="7">
-        <v>0.61563201964861403</v>
+        <v>-1.0874593121062599</v>
       </c>
       <c r="F16" s="9">
-        <v>3.0435736681849901E-2</v>
+        <v>1.4174868650294201E-2</v>
       </c>
       <c r="G16" s="7">
-        <v>49.438196374551403</v>
+        <v>13.034849665169901</v>
       </c>
       <c r="H16" s="2">
         <v>1</v>
       </c>
       <c r="I16" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="J16" s="4"/>
+        <v>48</v>
+      </c>
+      <c r="J16" s="4" t="s">
+        <v>49</v>
+      </c>
       <c r="K16" s="5" t="s">
-        <v>86</v>
+        <v>50</v>
       </c>
     </row>
     <row r="17" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C17" s="7">
         <v>135.46160097665</v>
       </c>
       <c r="D17" s="7">
-        <v>129.981851512752</v>
+        <v>136.07723299629799</v>
       </c>
       <c r="E17" s="7">
-        <v>-5.4797494638982798</v>
+        <v>0.61563201964861403</v>
       </c>
       <c r="F17" s="9">
-        <v>0.73663730461538401</v>
+        <v>2.0889809147941901E-2</v>
       </c>
       <c r="G17" s="7">
-        <v>134.42901166713901</v>
+        <v>-33.932297998186002</v>
       </c>
       <c r="H17" s="2">
         <v>1</v>
       </c>
       <c r="I17" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="J17" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="K17" s="4" t="s">
-        <v>54</v>
+        <v>81</v>
+      </c>
+      <c r="J17" s="4"/>
+      <c r="K17" s="5" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="18" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
-        <v>92</v>
+        <v>28</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>9</v>
+        <v>29</v>
       </c>
       <c r="C18" s="7">
         <v>135.46160097665</v>
       </c>
       <c r="D18" s="7">
-        <v>130.307543278781</v>
+        <v>129.981851512752</v>
       </c>
       <c r="E18" s="7">
-        <v>-5.1540576978685504</v>
+        <v>-5.4797494638982798</v>
       </c>
       <c r="F18" s="9">
-        <v>3.8655432734014297E-2</v>
+        <v>0.73663730461538401</v>
       </c>
       <c r="G18" s="7">
-        <v>7.50000000000004</v>
+        <v>134.42901166713901</v>
       </c>
       <c r="H18" s="2">
         <v>1</v>
       </c>
       <c r="I18" s="3" t="s">
-        <v>55</v>
+        <v>71</v>
       </c>
       <c r="J18" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="K18" s="5" t="s">
-        <v>57</v>
+        <v>53</v>
+      </c>
+      <c r="K18" s="4" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="19" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
-        <v>30</v>
+        <v>93</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>31</v>
+        <v>9</v>
       </c>
       <c r="C19" s="7">
         <v>135.46160097665</v>
       </c>
       <c r="D19" s="7">
-        <v>133.462247729079</v>
+        <v>130.307543278781</v>
       </c>
       <c r="E19" s="7">
-        <v>-1.9993532475706099</v>
+        <v>-5.1540576978685504</v>
       </c>
       <c r="F19" s="9">
-        <v>9.8011576103582396E-2</v>
+        <v>3.8655432734014297E-2</v>
       </c>
       <c r="G19" s="7">
-        <v>49.021640484329097</v>
+        <v>7.50000000000004</v>
       </c>
       <c r="H19" s="2">
         <v>1</v>
       </c>
       <c r="I19" s="3" t="s">
-        <v>80</v>
+        <v>55</v>
       </c>
       <c r="J19" s="4" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="K19" s="5" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
     </row>
     <row r="20" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>10</v>
+        <v>31</v>
       </c>
       <c r="C20" s="7">
         <v>135.46160097665</v>
       </c>
       <c r="D20" s="7">
-        <v>122.564472430718</v>
+        <v>133.462247729079</v>
       </c>
       <c r="E20" s="7">
-        <v>-12.8971285459314</v>
+        <v>-1.9993532475706099</v>
       </c>
       <c r="F20" s="9">
-        <v>-0.62178853607099305</v>
+        <v>9.8011576103582396E-2</v>
       </c>
       <c r="G20" s="7">
-        <v>-48.211393245913001</v>
+        <v>49.021640484329097</v>
       </c>
       <c r="H20" s="2">
         <v>1</v>
       </c>
       <c r="I20" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="J20" s="4"/>
+        <v>79</v>
+      </c>
+      <c r="J20" s="4" t="s">
+        <v>51</v>
+      </c>
       <c r="K20" s="5" t="s">
-        <v>88</v>
+        <v>52</v>
       </c>
     </row>
     <row r="21" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
-        <v>93</v>
+        <v>32</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>27</v>
+        <v>10</v>
       </c>
       <c r="C21" s="7">
         <v>135.46160097665</v>
       </c>
       <c r="D21" s="7">
-        <v>134.94181142571699</v>
+        <v>131.49325373174801</v>
       </c>
       <c r="E21" s="7">
-        <v>-0.51978955093250001</v>
+        <v>-3.9683472449019899</v>
       </c>
       <c r="F21" s="9">
-        <v>0.30611215582963103</v>
+        <v>0.62178583333929904</v>
       </c>
       <c r="G21" s="7">
-        <v>588.91556261657695</v>
+        <v>156.68634697683899</v>
       </c>
       <c r="H21" s="2">
         <v>1</v>
       </c>
-      <c r="I21" s="2" t="s">
-        <v>96</v>
-      </c>
+      <c r="I21" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="J21" s="4"/>
       <c r="K21" s="5" t="s">
-        <v>97</v>
+        <v>83</v>
       </c>
     </row>
     <row r="22" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>27</v>
+        <v>76</v>
       </c>
       <c r="C22" s="7">
         <v>135.46160097665</v>
       </c>
       <c r="D22" s="7">
-        <v>139.44086829482501</v>
+        <v>130.307543278781</v>
       </c>
       <c r="E22" s="7">
-        <v>3.9792673181751699</v>
+        <v>-5.1540576978685504</v>
       </c>
       <c r="F22" s="9">
-        <v>0.43078919998884702</v>
+        <v>0.68922045384102404</v>
       </c>
       <c r="G22" s="7">
-        <v>108.258421850985</v>
+        <v>133.72385298015701</v>
       </c>
       <c r="H22" s="2">
         <v>1</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="K22" s="5" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
     </row>
     <row r="23" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A23" s="2" t="s">
-        <v>91</v>
+        <v>77</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C23" s="7">
         <v>135.46160097665</v>
       </c>
       <c r="D23" s="7">
-        <v>124.569881234536</v>
+        <v>132.818331729742</v>
       </c>
       <c r="E23" s="7">
-        <v>-10.8917197421142</v>
+        <v>-2.6432692469078001</v>
       </c>
       <c r="F23" s="9">
-        <v>0.89034922155516405</v>
+        <v>0.58277686938970297</v>
       </c>
       <c r="G23" s="7">
-        <v>81.745513347402195</v>
+        <v>220.47578772819099</v>
+      </c>
+      <c r="H23" s="2">
+        <v>1</v>
+      </c>
+      <c r="I23" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="K23" s="5" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="24" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>77</v>
+        <v>27</v>
       </c>
       <c r="C24" s="7">
         <v>135.46160097665</v>
       </c>
       <c r="D24" s="7">
-        <v>132.818331729742</v>
+        <v>134.94181142571699</v>
       </c>
       <c r="E24" s="7">
-        <v>-2.6432692469078001</v>
+        <v>-0.51978955093250001</v>
       </c>
       <c r="F24" s="9">
-        <v>1.9209250919660501</v>
+        <v>0.31240814519386101</v>
       </c>
       <c r="G24" s="7">
-        <v>726.72320241807495</v>
+        <v>601.02813654757301</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A25" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C25" s="7">
+        <v>135.46160097665</v>
+      </c>
+      <c r="D25" s="7">
+        <v>139.44086829482501</v>
+      </c>
+      <c r="E25" s="7">
+        <v>3.9792673181751699</v>
+      </c>
+      <c r="F25" s="9">
+        <v>-0.904109084417827</v>
+      </c>
+      <c r="G25" s="7">
+        <v>227.20491289648601</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K20" xr:uid="{D3910A4A-016A-C04F-9DC6-2D7CC5B9E4C9}"/>
+  <autoFilter ref="A1:K21" xr:uid="{D3910A4A-016A-C04F-9DC6-2D7CC5B9E4C9}"/>
   <hyperlinks>
-    <hyperlink ref="K3" r:id="rId1" tooltip="Global Mitigation of Non-CO2 Greenhouse Gases: Landfills" display="https://19january2017snapshot.epa.gov/global-mitigation-non-co2-greenhouse-gases/global-mitigation-non-co2-greenhouse-gases-landfills_.html?utm_source=chatgpt.com" xr:uid="{1B17F12D-735D-2349-9BDA-CF3716E34838}"/>
-    <hyperlink ref="K12" r:id="rId2" tooltip="Global Mitigation of Non-CO2 Greenhouse Gases: Landfills" display="https://19january2017snapshot.epa.gov/global-mitigation-non-co2-greenhouse-gases/global-mitigation-non-co2-greenhouse-gases-landfills_.html?utm_source=chatgpt.com" xr:uid="{C86EF60A-BF47-5543-A8D0-C3E94136E596}"/>
-    <hyperlink ref="K18" r:id="rId3" tooltip="Landfills (PDF)" display="https://www.epa.gov/sites/default/files/2015-12/documents/landfills.pdf?utm_source=chatgpt.com" xr:uid="{E25157E3-1558-3D46-9F98-C2BFA7C7F40C}"/>
-    <hyperlink ref="K14" r:id="rId4" tooltip="Reduce Food Loss &amp; Waste" display="https://drawdown.org/explorer/reduce-food-loss-waste?utm_source=chatgpt.com" xr:uid="{C278F39D-9E38-EC4B-842E-31C1080F843A}"/>
-    <hyperlink ref="K15" r:id="rId5" tooltip="Nitric and Adipic Acid Production | Global Mitigation of Non ..." display="https://19january2017snapshot.epa.gov/global-mitigation-non-co2-greenhouse-gases/global-mitigation-non-co2-greenhouse-gases-nitric-and_.html?utm_source=chatgpt.com" xr:uid="{D83C1AAA-A906-8245-86EA-8269668F8040}"/>
-    <hyperlink ref="K6" r:id="rId6" tooltip="Reduce Food Loss &amp; Waste" display="https://drawdown.org/explorer/reduce-food-loss-waste?utm_source=chatgpt.com" xr:uid="{445AF596-8C8B-BA44-8F9A-A407F0699EC7}"/>
-    <hyperlink ref="K19" r:id="rId7" tooltip="A global analysis of the cost-efficiency of forest carbon ..." display="https://www.oecd.org/content/dam/oecd/en/publications/reports/2021/11/a-global-analysis-of-the-cost-efficiency-of-forest-carbon-sequestration_3ab6bef0/e4d45973-en.pdf?utm_source=chatgpt.com" xr:uid="{171188FE-2AFA-C740-9C96-E7CA42FF7002}"/>
-    <hyperlink ref="K20" r:id="rId8" xr:uid="{52E19A5C-B6B6-D14B-BFE1-D92A71AD17E7}"/>
-    <hyperlink ref="K4" r:id="rId9" xr:uid="{53F46158-0C98-CD4B-A7DC-A11369E624B1}"/>
-    <hyperlink ref="K7" r:id="rId10" xr:uid="{960EB68E-3EE1-D143-A55E-D40C01979E70}"/>
-    <hyperlink ref="K9" r:id="rId11" tooltip="Global Mitigation of Non-CO2 Greenhouse Gases" display="https://www.epa.gov/sites/default/files/2016-06/documents/mac_report_2013.pdf?utm_source=chatgpt.com" xr:uid="{4FDC818B-974D-FE4B-A304-1056093A0E1E}"/>
-    <hyperlink ref="K10" r:id="rId12" tooltip="Global Mitigation of Non-CO2 Greenhouse Gases" display="https://www.epa.gov/sites/default/files/2016-06/documents/mac_report_2013.pdf?utm_source=chatgpt.com" xr:uid="{FD662A82-0208-454F-8DE8-21322CB5B26A}"/>
-    <hyperlink ref="K11" r:id="rId13" tooltip="_x000a_            A perspective on methodologies and system boundaries to develop abatement cost for on-farm anaerobic digestion - PMC_x000a_        " display="https://pmc.ncbi.nlm.nih.gov/articles/PMC10506441/" xr:uid="{08A713B9-8809-C045-BBC4-D3858FAB9D4C}"/>
-    <hyperlink ref="K13" r:id="rId14" tooltip="_x000a_            A perspective on methodologies and system boundaries to develop abatement cost for on-farm anaerobic digestion - PMC_x000a_        " display="https://pmc.ncbi.nlm.nih.gov/articles/PMC10506441/" xr:uid="{8708EAAA-B421-1345-A662-56D780F47BF1}"/>
-    <hyperlink ref="K5" r:id="rId15" tooltip="Marginal Abatement Cost Curves for Greenhouse Gas ..." display="https://www.usda.gov/sites/default/files/documents/Marginal-Abatement-Cost-Curve-Estimate-Methodology-Report.pdf?utm_source=chatgpt.com" xr:uid="{10B6BF0C-2CFC-FA42-96F8-D82CEB599D83}"/>
-    <hyperlink ref="K8" r:id="rId16" tooltip="Waste Management" display="https://www.ipcc.ch/site/assets/uploads/2018/02/ar4-wg3-chapter10-1.pdf?utm_source=chatgpt.com" xr:uid="{0879220E-65A5-5645-8563-F9E061BD99E7}"/>
-    <hyperlink ref="K2" r:id="rId17" tooltip="AR4 WGIII Chapter 10: Waste management - 10.4.7 Waste management and mitigation costs and potentials" display="https://archive.ipcc.ch/publications_and_data/ar4/wg3/en/ch10-ens10-4-7.html" xr:uid="{2C151BAC-95DA-DF43-9144-1623C6D5E3D4}"/>
-    <hyperlink ref="K16" r:id="rId18" xr:uid="{6D459E53-FC67-8141-ACBD-945F093B7F62}"/>
-    <hyperlink ref="K21" r:id="rId19" xr:uid="{159C6FBE-D302-F447-9D34-A73F001C5F1F}"/>
-    <hyperlink ref="K22" r:id="rId20" xr:uid="{E4B833C9-E00F-A742-9145-3749662B217C}"/>
+    <hyperlink ref="K4" r:id="rId1" tooltip="Global Mitigation of Non-CO2 Greenhouse Gases: Landfills" display="https://19january2017snapshot.epa.gov/global-mitigation-non-co2-greenhouse-gases/global-mitigation-non-co2-greenhouse-gases-landfills_.html?utm_source=chatgpt.com" xr:uid="{1B17F12D-735D-2349-9BDA-CF3716E34838}"/>
+    <hyperlink ref="K13" r:id="rId2" tooltip="Global Mitigation of Non-CO2 Greenhouse Gases: Landfills" display="https://19january2017snapshot.epa.gov/global-mitigation-non-co2-greenhouse-gases/global-mitigation-non-co2-greenhouse-gases-landfills_.html?utm_source=chatgpt.com" xr:uid="{C86EF60A-BF47-5543-A8D0-C3E94136E596}"/>
+    <hyperlink ref="K19" r:id="rId3" tooltip="Landfills (PDF)" display="https://www.epa.gov/sites/default/files/2015-12/documents/landfills.pdf?utm_source=chatgpt.com" xr:uid="{E25157E3-1558-3D46-9F98-C2BFA7C7F40C}"/>
+    <hyperlink ref="K15" r:id="rId4" tooltip="Reduce Food Loss &amp; Waste" display="https://drawdown.org/explorer/reduce-food-loss-waste?utm_source=chatgpt.com" xr:uid="{C278F39D-9E38-EC4B-842E-31C1080F843A}"/>
+    <hyperlink ref="K16" r:id="rId5" tooltip="Nitric and Adipic Acid Production | Global Mitigation of Non ..." display="https://19january2017snapshot.epa.gov/global-mitigation-non-co2-greenhouse-gases/global-mitigation-non-co2-greenhouse-gases-nitric-and_.html?utm_source=chatgpt.com" xr:uid="{D83C1AAA-A906-8245-86EA-8269668F8040}"/>
+    <hyperlink ref="K7" r:id="rId6" tooltip="Reduce Food Loss &amp; Waste" display="https://drawdown.org/explorer/reduce-food-loss-waste?utm_source=chatgpt.com" xr:uid="{445AF596-8C8B-BA44-8F9A-A407F0699EC7}"/>
+    <hyperlink ref="K20" r:id="rId7" tooltip="A global analysis of the cost-efficiency of forest carbon ..." display="https://www.oecd.org/content/dam/oecd/en/publications/reports/2021/11/a-global-analysis-of-the-cost-efficiency-of-forest-carbon-sequestration_3ab6bef0/e4d45973-en.pdf?utm_source=chatgpt.com" xr:uid="{171188FE-2AFA-C740-9C96-E7CA42FF7002}"/>
+    <hyperlink ref="K21" r:id="rId8" xr:uid="{52E19A5C-B6B6-D14B-BFE1-D92A71AD17E7}"/>
+    <hyperlink ref="K5" r:id="rId9" xr:uid="{53F46158-0C98-CD4B-A7DC-A11369E624B1}"/>
+    <hyperlink ref="K8" r:id="rId10" xr:uid="{960EB68E-3EE1-D143-A55E-D40C01979E70}"/>
+    <hyperlink ref="K10" r:id="rId11" tooltip="Global Mitigation of Non-CO2 Greenhouse Gases" display="https://www.epa.gov/sites/default/files/2016-06/documents/mac_report_2013.pdf?utm_source=chatgpt.com" xr:uid="{4FDC818B-974D-FE4B-A304-1056093A0E1E}"/>
+    <hyperlink ref="K11" r:id="rId12" tooltip="Global Mitigation of Non-CO2 Greenhouse Gases" display="https://www.epa.gov/sites/default/files/2016-06/documents/mac_report_2013.pdf?utm_source=chatgpt.com" xr:uid="{FD662A82-0208-454F-8DE8-21322CB5B26A}"/>
+    <hyperlink ref="K12" r:id="rId13" tooltip="_x000a_            A perspective on methodologies and system boundaries to develop abatement cost for on-farm anaerobic digestion - PMC_x000a_        " display="https://pmc.ncbi.nlm.nih.gov/articles/PMC10506441/" xr:uid="{08A713B9-8809-C045-BBC4-D3858FAB9D4C}"/>
+    <hyperlink ref="K14" r:id="rId14" tooltip="_x000a_            A perspective on methodologies and system boundaries to develop abatement cost for on-farm anaerobic digestion - PMC_x000a_        " display="https://pmc.ncbi.nlm.nih.gov/articles/PMC10506441/" xr:uid="{8708EAAA-B421-1345-A662-56D780F47BF1}"/>
+    <hyperlink ref="K6" r:id="rId15" tooltip="Marginal Abatement Cost Curves for Greenhouse Gas ..." display="https://www.usda.gov/sites/default/files/documents/Marginal-Abatement-Cost-Curve-Estimate-Methodology-Report.pdf?utm_source=chatgpt.com" xr:uid="{10B6BF0C-2CFC-FA42-96F8-D82CEB599D83}"/>
+    <hyperlink ref="K9" r:id="rId16" tooltip="Waste Management" display="https://www.ipcc.ch/site/assets/uploads/2018/02/ar4-wg3-chapter10-1.pdf?utm_source=chatgpt.com" xr:uid="{0879220E-65A5-5645-8563-F9E061BD99E7}"/>
+    <hyperlink ref="K3" r:id="rId17" tooltip="AR4 WGIII Chapter 10: Waste management - 10.4.7 Waste management and mitigation costs and potentials" display="https://archive.ipcc.ch/publications_and_data/ar4/wg3/en/ch10-ens10-4-7.html" xr:uid="{2C151BAC-95DA-DF43-9144-1623C6D5E3D4}"/>
+    <hyperlink ref="K17" r:id="rId18" xr:uid="{6D459E53-FC67-8141-ACBD-945F093B7F62}"/>
+    <hyperlink ref="K22" r:id="rId19" xr:uid="{159C6FBE-D302-F447-9D34-A73F001C5F1F}"/>
+    <hyperlink ref="K23" r:id="rId20" xr:uid="{E4B833C9-E00F-A742-9145-3749662B217C}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>